<commit_message>
Importación masiva: un solo error de sucursal por fila y planilla de ejemplo con EAN válidos
</commit_message>
<xml_diff>
--- a/docs/examples/importacion-ejemplo.xlsx
+++ b/docs/examples/importacion-ejemplo.xlsx
@@ -98,7 +98,7 @@
     <t>L2410B</t>
   </si>
   <si>
-    <t>7798877000015</t>
+    <t>7798877000010</t>
   </si>
   <si>
     <t>Arroz largo fino Gran Espiga 1 kg</t>
@@ -125,7 +125,7 @@
     <t/>
   </si>
   <si>
-    <t>7798877000022</t>
+    <t>7798877000027</t>
   </si>
   <si>
     <t>Sin Marca</t>
@@ -140,7 +140,7 @@
     <t>480</t>
   </si>
   <si>
-    <t>7798877000039</t>
+    <t>7798877000034</t>
   </si>
   <si>
     <t>Fideos guiseros Doña Rosa 500 g</t>
@@ -161,7 +161,7 @@
     <t>mil doscientos</t>
   </si>
   <si>
-    <t>7798877000046</t>
+    <t>7798877000041</t>
   </si>
   <si>
     <t>Aceite de girasol Solcito 900 ml</t>
@@ -179,7 +179,7 @@
     <t>12,5</t>
   </si>
   <si>
-    <t>7798877000053</t>
+    <t>7798877000058</t>
   </si>
   <si>
     <t>Yogur firme durazno Vaquita 190 g</t>
@@ -197,7 +197,7 @@
     <t>31/02/2027</t>
   </si>
   <si>
-    <t>7798877000060</t>
+    <t>7798877000065</t>
   </si>
   <si>
     <t>Galletitas dulces Ronda 300 g</t>
@@ -233,7 +233,7 @@
     <t>M2408</t>
   </si>
   <si>
-    <t>7798877000085</t>
+    <t>7798877000089</t>
   </si>
   <si>
     <t>Cafe molido Aroma del Norte 250 g</t>
@@ -251,7 +251,7 @@
     <t>3.200</t>
   </si>
   <si>
-    <t>7798877000092</t>
+    <t>7798877000096</t>
   </si>
   <si>
     <t>Hamburguesas de carne Pampa 4 u</t>
@@ -278,7 +278,7 @@
     <t>Sucursal Norte</t>
   </si>
   <si>
-    <t>7798877000108</t>
+    <t>7798877000102</t>
   </si>
   <si>
     <t>Queso cremoso La Tranquera 500 g</t>
@@ -293,7 +293,7 @@
     <t>Q2312</t>
   </si>
   <si>
-    <t>7798877000115</t>
+    <t>7798877000119</t>
   </si>
   <si>
     <t>Azucar comun Dulce Sol 1 kg</t>
@@ -308,7 +308,7 @@
     <t>1.290</t>
   </si>
   <si>
-    <t>7798877000122</t>
+    <t>7798877000126</t>
   </si>
   <si>
     <t>Agua mineral Vertiente 2 L</t>
@@ -332,7 +332,7 @@
     <t>980</t>
   </si>
   <si>
-    <t>7798877000139</t>
+    <t>7798877000133</t>
   </si>
   <si>
     <t>Jugo en polvo naranja Solcito 20 g</t>
@@ -344,7 +344,7 @@
     <t>320</t>
   </si>
   <si>
-    <t>7798877000146</t>
+    <t>7798877000140</t>
   </si>
   <si>
     <t>Fideos tirabuzon Dona Rosa 500 g</t>
@@ -353,7 +353,7 @@
     <t>870</t>
   </si>
   <si>
-    <t>7798877000153</t>
+    <t>7798877000157</t>
   </si>
   <si>
     <t>Manteca La Tranquera 200 g</t>
@@ -368,7 +368,7 @@
     <t>MT2410</t>
   </si>
   <si>
-    <t>7798877000160</t>
+    <t>7798877000164</t>
   </si>
   <si>
     <t>Pan rallado Crocantes 500 g</t>

</xml_diff>